<commit_message>
Update developer-di-practitioner from the Content Editor
</commit_message>
<xml_diff>
--- a/developer-di-practitioner/10-mod3-excel-writer/files/Sales_and_Expenses_2017.xlsx
+++ b/developer-di-practitioner/10-mod3-excel-writer/files/Sales_and_Expenses_2017.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sales Chart" r:id="rId1" sheetId="4"/>
     <sheet name="SourceData" r:id="rId2" sheetId="1"/>
   </sheets>
-  <calcPr calcId="171027" concurrentCalc="0"/>
+  <calcPr fullCalcOnLoad="1" calcId="171027" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="http://schemas.microsoft.com/office/mac/excel/2008/main">
       <mx:ArchID Flags="2"/>
@@ -3113,7 +3113,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="6" t="n">
-        <f ref="B10:G10" si="4" t="shared">B5+B6+B8</f>
+        <f ref="B10:G10" si="4" t="shared">SUM(B5:B8)</f>
         <v>35655.55</v>
       </c>
       <c r="C10" s="6" t="n">

</xml_diff>